<commit_message>
- Temperatures.xslsx fixed to have static values  - excel sheet update now works as intended in the answer
</commit_message>
<xml_diff>
--- a/Introductory/Homeworks/Temperatures.xlsx
+++ b/Introductory/Homeworks/Temperatures.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\tis254\Documents\Python-Software-Carpentry\Introductory\Homeworks\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9D352243-8E8F-47DA-BA60-C1A8331A97CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B455F3F0-D90D-46FE-8167-C7F6E5602710}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -515,12 +515,10 @@
         <v>5</v>
       </c>
       <c r="B2">
-        <f ca="1">RANDBETWEEN(13,41.5)</f>
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="C2" s="1">
-        <f ca="1">RANDBETWEEN(DATE(2020,2,14),DATE(2026,7,22))</f>
-        <v>44563</v>
+        <v>44281</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -528,12 +526,10 @@
         <v>6</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B22" ca="1" si="0">RANDBETWEEN(13,41.5)</f>
-        <v>27</v>
+        <v>41</v>
       </c>
       <c r="C3" s="1">
-        <f t="shared" ref="C3:C22" ca="1" si="1">RANDBETWEEN(DATE(2020,2,14),DATE(2026,7,22))</f>
-        <v>45369</v>
+        <v>43894</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -541,12 +537,10 @@
         <v>7</v>
       </c>
       <c r="B4">
-        <f t="shared" ca="1" si="0"/>
-        <v>28</v>
+        <v>22</v>
       </c>
       <c r="C4" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>46086</v>
+        <v>44698</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -554,12 +548,10 @@
         <v>8</v>
       </c>
       <c r="B5">
-        <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>30</v>
       </c>
       <c r="C5" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45939</v>
+        <v>45578</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -567,12 +559,10 @@
         <v>9</v>
       </c>
       <c r="B6">
-        <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C6" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>43898</v>
+        <v>46128</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -580,12 +570,10 @@
         <v>10</v>
       </c>
       <c r="B7">
-        <f t="shared" ca="1" si="0"/>
-        <v>38</v>
+        <v>15</v>
       </c>
       <c r="C7" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45090</v>
+        <v>44502</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -593,12 +581,10 @@
         <v>11</v>
       </c>
       <c r="B8">
-        <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>21</v>
       </c>
       <c r="C8" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44113</v>
+        <v>43938</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -606,12 +592,10 @@
         <v>12</v>
       </c>
       <c r="B9">
-        <f t="shared" ca="1" si="0"/>
-        <v>29</v>
+        <v>17</v>
       </c>
       <c r="C9" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45850</v>
+        <v>45365</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -619,12 +603,10 @@
         <v>13</v>
       </c>
       <c r="B10">
-        <f t="shared" ca="1" si="0"/>
-        <v>41</v>
+        <v>16</v>
       </c>
       <c r="C10" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45889</v>
+        <v>43893</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -632,12 +614,10 @@
         <v>14</v>
       </c>
       <c r="B11">
-        <f t="shared" ca="1" si="0"/>
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C11" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>43888</v>
+        <v>44885</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -645,12 +625,10 @@
         <v>15</v>
       </c>
       <c r="B12">
-        <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>30</v>
       </c>
       <c r="C12" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44649</v>
+        <v>44596</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -658,12 +636,10 @@
         <v>16</v>
       </c>
       <c r="B13">
-        <f t="shared" ca="1" si="0"/>
-        <v>29</v>
+        <v>18</v>
       </c>
       <c r="C13" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45844</v>
+        <v>45936</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -671,12 +647,10 @@
         <v>17</v>
       </c>
       <c r="B14">
-        <f t="shared" ca="1" si="0"/>
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="C14" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44026</v>
+        <v>45702</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
@@ -684,12 +658,10 @@
         <v>18</v>
       </c>
       <c r="B15">
-        <f t="shared" ca="1" si="0"/>
-        <v>16</v>
+        <v>14</v>
       </c>
       <c r="C15" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45052</v>
+        <v>45724</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -697,12 +669,10 @@
         <v>19</v>
       </c>
       <c r="B16">
-        <f t="shared" ca="1" si="0"/>
-        <v>36</v>
+        <v>22</v>
       </c>
       <c r="C16" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44094</v>
+        <v>45486</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
@@ -710,12 +680,10 @@
         <v>20</v>
       </c>
       <c r="B17">
-        <f t="shared" ca="1" si="0"/>
-        <v>20</v>
+        <v>37</v>
       </c>
       <c r="C17" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45182</v>
+        <v>45270</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
@@ -723,12 +691,10 @@
         <v>21</v>
       </c>
       <c r="B18">
-        <f t="shared" ca="1" si="0"/>
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="C18" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44589</v>
+        <v>44032</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -736,12 +702,10 @@
         <v>22</v>
       </c>
       <c r="B19">
-        <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>25</v>
       </c>
       <c r="C19" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44808</v>
+        <v>45195</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -749,12 +713,10 @@
         <v>23</v>
       </c>
       <c r="B20">
-        <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>40</v>
       </c>
       <c r="C20" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44015</v>
+        <v>45557</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -762,12 +724,10 @@
         <v>24</v>
       </c>
       <c r="B21">
-        <f t="shared" ca="1" si="0"/>
-        <v>35</v>
+        <v>31</v>
       </c>
       <c r="C21" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45321</v>
+        <v>45955</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -775,12 +735,10 @@
         <v>25</v>
       </c>
       <c r="B22">
-        <f t="shared" ca="1" si="0"/>
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C22" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45510</v>
+        <v>44893</v>
       </c>
     </row>
   </sheetData>
@@ -812,12 +770,10 @@
         <v>26</v>
       </c>
       <c r="B2">
-        <f ca="1">RANDBETWEEN(13,41.5)</f>
-        <v>24</v>
+        <v>39</v>
       </c>
       <c r="C2" s="1">
-        <f ca="1">RANDBETWEEN(DATE(2020,2,14),DATE(2026,7,22))</f>
-        <v>44333</v>
+        <v>44502</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.35">
@@ -825,12 +781,10 @@
         <v>27</v>
       </c>
       <c r="B3">
-        <f t="shared" ref="B3:B22" ca="1" si="0">RANDBETWEEN(13,41.5)</f>
-        <v>35</v>
+        <v>13</v>
       </c>
       <c r="C3" s="1">
-        <f t="shared" ref="C3:C22" ca="1" si="1">RANDBETWEEN(DATE(2020,2,14),DATE(2026,7,22))</f>
-        <v>44839</v>
+        <v>44920</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.35">
@@ -838,12 +792,10 @@
         <v>28</v>
       </c>
       <c r="B4">
-        <f t="shared" ca="1" si="0"/>
-        <v>18</v>
+        <v>32</v>
       </c>
       <c r="C4" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45067</v>
+        <v>44973</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.35">
@@ -851,12 +803,10 @@
         <v>29</v>
       </c>
       <c r="B5">
-        <f t="shared" ca="1" si="0"/>
-        <v>33</v>
+        <v>36</v>
       </c>
       <c r="C5" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>46041</v>
+        <v>45698</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.35">
@@ -864,12 +814,10 @@
         <v>30</v>
       </c>
       <c r="B6">
-        <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>28</v>
       </c>
       <c r="C6" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44716</v>
+        <v>44127</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.35">
@@ -877,12 +825,10 @@
         <v>31</v>
       </c>
       <c r="B7">
-        <f t="shared" ca="1" si="0"/>
-        <v>23</v>
+        <v>14</v>
       </c>
       <c r="C7" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45388</v>
+        <v>44052</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.35">
@@ -890,12 +836,10 @@
         <v>32</v>
       </c>
       <c r="B8">
-        <f t="shared" ca="1" si="0"/>
-        <v>19</v>
+        <v>37</v>
       </c>
       <c r="C8" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45869</v>
+        <v>44875</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.35">
@@ -903,12 +847,10 @@
         <v>33</v>
       </c>
       <c r="B9">
-        <f t="shared" ca="1" si="0"/>
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="C9" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45549</v>
+        <v>46195</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.35">
@@ -916,12 +858,10 @@
         <v>34</v>
       </c>
       <c r="B10">
-        <f t="shared" ca="1" si="0"/>
-        <v>27</v>
+        <v>38</v>
       </c>
       <c r="C10" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44379</v>
+        <v>45578</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.35">
@@ -929,12 +869,10 @@
         <v>35</v>
       </c>
       <c r="B11">
-        <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C11" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45947</v>
+        <v>44155</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.35">
@@ -942,12 +880,10 @@
         <v>15</v>
       </c>
       <c r="B12">
-        <f t="shared" ca="1" si="0"/>
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C12" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44440</v>
+        <v>45460</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.35">
@@ -955,12 +891,10 @@
         <v>36</v>
       </c>
       <c r="B13">
-        <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C13" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44466</v>
+        <v>44418</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.35">
@@ -968,12 +902,10 @@
         <v>37</v>
       </c>
       <c r="B14">
-        <f t="shared" ca="1" si="0"/>
-        <v>28</v>
+        <v>18</v>
       </c>
       <c r="C14" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44239</v>
+        <v>45612</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.35">
@@ -981,12 +913,10 @@
         <v>38</v>
       </c>
       <c r="B15">
-        <f t="shared" ca="1" si="0"/>
-        <v>26</v>
+        <v>16</v>
       </c>
       <c r="C15" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44976</v>
+        <v>45788</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.35">
@@ -994,12 +924,10 @@
         <v>39</v>
       </c>
       <c r="B16">
-        <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="C16" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45897</v>
+        <v>46145</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.35">
@@ -1007,12 +935,10 @@
         <v>40</v>
       </c>
       <c r="B17">
-        <f t="shared" ca="1" si="0"/>
-        <v>35</v>
+        <v>29</v>
       </c>
       <c r="C17" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45898</v>
+        <v>44950</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.35">
@@ -1020,12 +946,10 @@
         <v>41</v>
       </c>
       <c r="B18">
-        <f t="shared" ca="1" si="0"/>
-        <v>40</v>
+        <v>29</v>
       </c>
       <c r="C18" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44919</v>
+        <v>44701</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.35">
@@ -1033,12 +957,10 @@
         <v>42</v>
       </c>
       <c r="B19">
-        <f t="shared" ca="1" si="0"/>
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C19" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>44295</v>
+        <v>44604</v>
       </c>
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.35">
@@ -1046,12 +968,10 @@
         <v>43</v>
       </c>
       <c r="B20">
-        <f t="shared" ca="1" si="0"/>
-        <v>14</v>
+        <v>26</v>
       </c>
       <c r="C20" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>45934</v>
+        <v>45813</v>
       </c>
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.35">
@@ -1059,12 +979,10 @@
         <v>44</v>
       </c>
       <c r="B21">
-        <f t="shared" ca="1" si="0"/>
-        <v>41</v>
+        <v>23</v>
       </c>
       <c r="C21" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>43973</v>
+        <v>46105</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.35">
@@ -1072,12 +990,10 @@
         <v>45</v>
       </c>
       <c r="B22">
-        <f t="shared" ca="1" si="0"/>
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="C22" s="1">
-        <f t="shared" ca="1" si="1"/>
-        <v>43905</v>
+        <v>44872</v>
       </c>
     </row>
   </sheetData>

</xml_diff>